<commit_message>
condprep_v1 eval results (server)
</commit_message>
<xml_diff>
--- a/results/metrics_all_arms.xlsx
+++ b/results/metrics_all_arms.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:V60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3088,6 +3088,1258 @@
         <v>0.6235138949706565</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>val</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0.6166191613417338</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.3852798038493804</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.2719114337900373</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.4831994562711893</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.4851714145284347</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.2180621727165611</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.4680545419406799</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.5370764128995205</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0.6295908999985338</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.7944000915224365</v>
+      </c>
+      <c r="P42" t="n">
+        <v>0.4757588795795645</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>0.646269522708613</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>val_clear</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0.5450199999999999</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.33603</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.33826</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.22289</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.41493</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.45756</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.17579</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.40897</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0.45704</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0.53327</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0.77738</v>
+      </c>
+      <c r="P43" t="n">
+        <v>0.3983</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>0.55911</v>
+      </c>
+      <c r="R43" t="n">
+        <v>0.17873</v>
+      </c>
+      <c r="S43" t="n">
+        <v>0.47339</v>
+      </c>
+      <c r="T43" t="n">
+        <v>0.44659</v>
+      </c>
+      <c r="U43" t="n">
+        <v>0.13947</v>
+      </c>
+      <c r="V43" t="n">
+        <v>0.45312</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>val_clear</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0.5750081960561718</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.3584674002902657</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.2236416855137549</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.4684935499116013</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.4651946719637915</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.1866892131163424</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.4483178809458384</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0.456187996000264</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0.6098883997384426</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0.7786071634088101</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0.4169838408206484</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>0.6133735803126941</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>val_dawndusk</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0.55824</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.36053</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.36712</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.24872</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.49267</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.49103</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0.10486</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.46538</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0.49151</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0.60862</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0.78991</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0.26099</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0.64016</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0.17803</v>
+      </c>
+      <c r="S45" t="n">
+        <v>0.56326</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0.5012</v>
+      </c>
+      <c r="U45" t="n">
+        <v>0.08316</v>
+      </c>
+      <c r="V45" t="n">
+        <v>0.50996</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>val_dawndusk</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0.5916112782175317</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.382030359647459</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.253270869042963</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.5408061619448677</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.5006882539949806</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.109112355624676</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0.5062741576298078</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0.5197583662513091</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0.6744188775239123</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.7935586444496625</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0.2869495976687248</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>0.6833709051940494</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>val_day</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0.54067</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.34228</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.35169</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.19129</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.40837</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0.50098</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0.18409</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0.42667</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0.41551</v>
+      </c>
+      <c r="N47" t="n">
+        <v>0.53147</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0.80049</v>
+      </c>
+      <c r="P47" t="n">
+        <v>0.36981</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>0.58609</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0.15837</v>
+      </c>
+      <c r="S47" t="n">
+        <v>0.45871</v>
+      </c>
+      <c r="T47" t="n">
+        <v>0.50737</v>
+      </c>
+      <c r="U47" t="n">
+        <v>0.17119</v>
+      </c>
+      <c r="V47" t="n">
+        <v>0.46284</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>val_day</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0.5710957813845023</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.3649669654786931</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.1927766290337872</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.4629682752485437</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.5107178090512239</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0.1983177533465205</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0.4600543607133903</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0.410571743224533</v>
+      </c>
+      <c r="N48" t="n">
+        <v>0.6099474891707019</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0.8054220525521628</v>
+      </c>
+      <c r="P48" t="n">
+        <v>0.3973968480793638</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>0.63214077389575</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>val_foggy</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0.6516</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.27379</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.22668</v>
+      </c>
+      <c r="H49" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.45502</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0.16634</v>
+      </c>
+      <c r="M49" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N49" t="n">
+        <v>-1</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0.74688</v>
+      </c>
+      <c r="P49" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>0.20792</v>
+      </c>
+      <c r="R49" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S49" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T49" t="n">
+        <v>0.47211</v>
+      </c>
+      <c r="U49" t="n">
+        <v>0</v>
+      </c>
+      <c r="V49" t="n">
+        <v>0.20792</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>val_foggy</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0.6612593344374345</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.2797599277535188</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0.4565702116270248</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0.1837095716335315</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0.7388077225170584</v>
+      </c>
+      <c r="P50" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0.2499702807952449</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>val_night</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0.55191</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.32742</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.31945</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.24771</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0.39652</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0.43053</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0.16758</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.39474</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0.50784</v>
+      </c>
+      <c r="N51" t="n">
+        <v>0.51376</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0.76207</v>
+      </c>
+      <c r="P51" t="n">
+        <v>0.42967</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0.5462</v>
+      </c>
+      <c r="R51" t="n">
+        <v>0.18736</v>
+      </c>
+      <c r="S51" t="n">
+        <v>0.44746</v>
+      </c>
+      <c r="T51" t="n">
+        <v>0.40897</v>
+      </c>
+      <c r="U51" t="n">
+        <v>0.11238</v>
+      </c>
+      <c r="V51" t="n">
+        <v>0.44109</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>val_night</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>0.5796638787229778</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.3491791106603472</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.251283209793608</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0.4403006780416179</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0.4366865941713659</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0.1760974960791905</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0.4415275752159535</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0.5072964487235589</v>
+      </c>
+      <c r="N52" t="n">
+        <v>0.5759651218858668</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0.7620743915621634</v>
+      </c>
+      <c r="P52" t="n">
+        <v>0.4421527334159612</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>0.6108306980273386</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>val_overcast</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0.56101</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.34494</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.34269</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.21757</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0.41935</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0.50719</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0.1442</v>
+      </c>
+      <c r="L53" t="n">
+        <v>0.43638</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0.49061</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0.54127</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0.8066</v>
+      </c>
+      <c r="P53" t="n">
+        <v>0.35574</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>0.61084</v>
+      </c>
+      <c r="R53" t="n">
+        <v>0.15986</v>
+      </c>
+      <c r="S53" t="n">
+        <v>0.471</v>
+      </c>
+      <c r="T53" t="n">
+        <v>0.51531</v>
+      </c>
+      <c r="U53" t="n">
+        <v>0.1036</v>
+      </c>
+      <c r="V53" t="n">
+        <v>0.46367</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>val_overcast</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0.5891248060707339</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.3644549235811377</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.2251484660889475</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0.4630131704740349</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0.5168818808697424</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0.1518640642930717</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0.4653670361798921</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.4942390565051479</v>
+      </c>
+      <c r="N54" t="n">
+        <v>0.6054102978677458</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0.8122846034166027</v>
+      </c>
+      <c r="P54" t="n">
+        <v>0.3916597809312669</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>0.6420302916329059</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>val_partlycloudy</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0.54911</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.36013</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.37823</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.19571</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0.44185</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0.49301</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.22938</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.44068</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0.39778</v>
+      </c>
+      <c r="N55" t="n">
+        <v>0.55396</v>
+      </c>
+      <c r="O55" t="n">
+        <v>0.79065</v>
+      </c>
+      <c r="P55" t="n">
+        <v>0.39664</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>0.60654</v>
+      </c>
+      <c r="R55" t="n">
+        <v>0.18647</v>
+      </c>
+      <c r="S55" t="n">
+        <v>0.50176</v>
+      </c>
+      <c r="T55" t="n">
+        <v>0.50324</v>
+      </c>
+      <c r="U55" t="n">
+        <v>0.23638</v>
+      </c>
+      <c r="V55" t="n">
+        <v>0.4633</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>val_partlycloudy</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0.5733275239901532</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.3806151135292942</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.1962743511297022</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0.4958794996016541</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.50172787756408</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.2350107173949731</v>
+      </c>
+      <c r="L56" t="n">
+        <v>0.4741831219560614</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0.38290087563408</v>
+      </c>
+      <c r="N56" t="n">
+        <v>0.6375577950390052</v>
+      </c>
+      <c r="O56" t="n">
+        <v>0.7945574213478279</v>
+      </c>
+      <c r="P56" t="n">
+        <v>0.4074859463902007</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>0.6441355815396514</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>val_rainy</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>0.55988</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.3593</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.3826</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.23941</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0.42403</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0.48462</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0.19756</v>
+      </c>
+      <c r="L57" t="n">
+        <v>0.45088</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0.50449</v>
+      </c>
+      <c r="N57" t="n">
+        <v>0.56532</v>
+      </c>
+      <c r="O57" t="n">
+        <v>0.78996</v>
+      </c>
+      <c r="P57" t="n">
+        <v>0.31355</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>0.6260599999999999</v>
+      </c>
+      <c r="R57" t="n">
+        <v>0.18197</v>
+      </c>
+      <c r="S57" t="n">
+        <v>0.46292</v>
+      </c>
+      <c r="T57" t="n">
+        <v>0.48544</v>
+      </c>
+      <c r="U57" t="n">
+        <v>0.28264</v>
+      </c>
+      <c r="V57" t="n">
+        <v>0.50005</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>val_rainy</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>0.5865980377874798</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.382020561552171</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.2378758229306403</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0.4907802933271057</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.4931700081551854</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0.1988132767646548</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0.4894634065832686</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0.4815664530856899</v>
+      </c>
+      <c r="N58" t="n">
+        <v>0.650270631055061</v>
+      </c>
+      <c r="O58" t="n">
+        <v>0.7908118049205728</v>
+      </c>
+      <c r="P58" t="n">
+        <v>0.3257716901581438</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>0.6845696097179315</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>val_snowy</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0.48025</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.31276</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.31568</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.1384</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0.35657</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0.48797</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0.1505</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0.43036</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0.3304</v>
+      </c>
+      <c r="N59" t="n">
+        <v>0.46295</v>
+      </c>
+      <c r="O59" t="n">
+        <v>0.79504</v>
+      </c>
+      <c r="P59" t="n">
+        <v>0.22772</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>0.58516</v>
+      </c>
+      <c r="R59" t="n">
+        <v>0.10723</v>
+      </c>
+      <c r="S59" t="n">
+        <v>0.38243</v>
+      </c>
+      <c r="T59" t="n">
+        <v>0.49165</v>
+      </c>
+      <c r="U59" t="n">
+        <v>0.11881</v>
+      </c>
+      <c r="V59" t="n">
+        <v>0.47829</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-17T10:35:41.993358+07:00</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>condprep_v1</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>val_snowy</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>0.5262351242700253</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.3399621689215517</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.1452873683250423</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0.3957616355150683</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.4986371537366154</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0.1884656509695291</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0.4716590360615037</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0.3447915749124503</v>
+      </c>
+      <c r="N60" t="n">
+        <v>0.5256999667638885</v>
+      </c>
+      <c r="O60" t="n">
+        <v>0.8007500514542626</v>
+      </c>
+      <c r="P60" t="n">
+        <v>0.3116377786571692</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>0.6482962495623558</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
run test result of all weather conditions
</commit_message>
<xml_diff>
--- a/results/metrics_all_arms.xlsx
+++ b/results/metrics_all_arms.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V60"/>
+  <dimension ref="A1:V84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4340,6 +4340,1590 @@
         <v>0.6482962495623558</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>val_clear</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>0.53987</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.33922</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.34562</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.21962</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0.41621</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0.46003</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0.19305</v>
+      </c>
+      <c r="L61" t="n">
+        <v>0.40718</v>
+      </c>
+      <c r="M61" t="n">
+        <v>0.42247</v>
+      </c>
+      <c r="N61" t="n">
+        <v>0.5371</v>
+      </c>
+      <c r="O61" t="n">
+        <v>0.77986</v>
+      </c>
+      <c r="P61" t="n">
+        <v>0.40921</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>0.5507</v>
+      </c>
+      <c r="R61" t="n">
+        <v>0.20682</v>
+      </c>
+      <c r="S61" t="n">
+        <v>0.46896</v>
+      </c>
+      <c r="T61" t="n">
+        <v>0.449</v>
+      </c>
+      <c r="U61" t="n">
+        <v>0.15085</v>
+      </c>
+      <c r="V61" t="n">
+        <v>0.45248</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>val_clear</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>0.5713017211912075</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.3612779139674622</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.2244580163955984</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0.4684513295268889</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0.4673631717563939</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0.198328584262968</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0.4477884678954617</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0.4302813186899345</v>
+      </c>
+      <c r="N62" t="n">
+        <v>0.6089120522137995</v>
+      </c>
+      <c r="O62" t="n">
+        <v>0.7817871810264223</v>
+      </c>
+      <c r="P62" t="n">
+        <v>0.4280921620212768</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>0.6074358920046048</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>val_foggy</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>0.64637</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.28078</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0.22642</v>
+      </c>
+      <c r="H63" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I63" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0.45521</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L63" t="n">
+        <v>0.18713</v>
+      </c>
+      <c r="M63" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N63" t="n">
+        <v>-1</v>
+      </c>
+      <c r="O63" t="n">
+        <v>0.73119</v>
+      </c>
+      <c r="P63" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>0.20792</v>
+      </c>
+      <c r="R63" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S63" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T63" t="n">
+        <v>0.47134</v>
+      </c>
+      <c r="U63" t="n">
+        <v>0</v>
+      </c>
+      <c r="V63" t="n">
+        <v>0.20792</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>val_foggy</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>0.6585389405866976</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.2895267873610702</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0.4639131380029432</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0.199</v>
+      </c>
+      <c r="L64" t="n">
+        <v>0.2056672240802676</v>
+      </c>
+      <c r="O64" t="n">
+        <v>0.7287606344691229</v>
+      </c>
+      <c r="P64" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>0.2518561872909699</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>val_overcast</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>0.55332</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.35025</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0.35713</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0.25124</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0.41918</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0.51039</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0.13628</v>
+      </c>
+      <c r="L65" t="n">
+        <v>0.43415</v>
+      </c>
+      <c r="M65" t="n">
+        <v>0.52395</v>
+      </c>
+      <c r="N65" t="n">
+        <v>0.53711</v>
+      </c>
+      <c r="O65" t="n">
+        <v>0.8110000000000001</v>
+      </c>
+      <c r="P65" t="n">
+        <v>0.29334</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>0.60119</v>
+      </c>
+      <c r="R65" t="n">
+        <v>0.22969</v>
+      </c>
+      <c r="S65" t="n">
+        <v>0.458</v>
+      </c>
+      <c r="T65" t="n">
+        <v>0.51772</v>
+      </c>
+      <c r="U65" t="n">
+        <v>0.11672</v>
+      </c>
+      <c r="V65" t="n">
+        <v>0.46353</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>val_overcast</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0.5925103159026186</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.3723709441918926</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0.249241200703151</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0.4709568613342354</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0.5191265833105385</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0.1558021407108336</v>
+      </c>
+      <c r="L66" t="n">
+        <v>0.4667279349007045</v>
+      </c>
+      <c r="M66" t="n">
+        <v>0.5075065460253489</v>
+      </c>
+      <c r="N66" t="n">
+        <v>0.6260656041249608</v>
+      </c>
+      <c r="O66" t="n">
+        <v>0.8148716321807958</v>
+      </c>
+      <c r="P66" t="n">
+        <v>0.3711711085979931</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>0.6429366885839947</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>val_partlycloudy</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>0.54222</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.35363</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0.36464</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0.17481</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0.43238</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0.4929</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0.22593</v>
+      </c>
+      <c r="L67" t="n">
+        <v>0.44213</v>
+      </c>
+      <c r="M67" t="n">
+        <v>0.34699</v>
+      </c>
+      <c r="N67" t="n">
+        <v>0.55991</v>
+      </c>
+      <c r="O67" t="n">
+        <v>0.79162</v>
+      </c>
+      <c r="P67" t="n">
+        <v>0.41312</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>0.59944</v>
+      </c>
+      <c r="R67" t="n">
+        <v>0.16797</v>
+      </c>
+      <c r="S67" t="n">
+        <v>0.48251</v>
+      </c>
+      <c r="T67" t="n">
+        <v>0.49806</v>
+      </c>
+      <c r="U67" t="n">
+        <v>0.21434</v>
+      </c>
+      <c r="V67" t="n">
+        <v>0.4603</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>val_partlycloudy</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>0.5653938868675076</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.3709874502740809</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0.1665156342255011</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0.4737899991762492</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0.5022270392537865</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0.2354622329557182</v>
+      </c>
+      <c r="L68" t="n">
+        <v>0.4769423457591497</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0.3392339187278756</v>
+      </c>
+      <c r="N68" t="n">
+        <v>0.6281842432961751</v>
+      </c>
+      <c r="O68" t="n">
+        <v>0.7949453261547628</v>
+      </c>
+      <c r="P68" t="n">
+        <v>0.4212735811281531</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>0.6433323650305713</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>val_rainy</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>0.57041</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.37009</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.38966</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.27739</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0.42465</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0.48633</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0.21724</v>
+      </c>
+      <c r="L69" t="n">
+        <v>0.44482</v>
+      </c>
+      <c r="M69" t="n">
+        <v>0.54165</v>
+      </c>
+      <c r="N69" t="n">
+        <v>0.55438</v>
+      </c>
+      <c r="O69" t="n">
+        <v>0.7900700000000001</v>
+      </c>
+      <c r="P69" t="n">
+        <v>0.34531</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>0.62065</v>
+      </c>
+      <c r="R69" t="n">
+        <v>0.26018</v>
+      </c>
+      <c r="S69" t="n">
+        <v>0.46359</v>
+      </c>
+      <c r="T69" t="n">
+        <v>0.48927</v>
+      </c>
+      <c r="U69" t="n">
+        <v>0.22512</v>
+      </c>
+      <c r="V69" t="n">
+        <v>0.5101599999999999</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>val_rainy</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0.5977286194595186</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.3872167447353814</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0.2682410975096839</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0.4782115950063095</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0.4958161701209158</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0.2044701508396868</v>
+      </c>
+      <c r="L70" t="n">
+        <v>0.4893447102003113</v>
+      </c>
+      <c r="M70" t="n">
+        <v>0.52249167710674</v>
+      </c>
+      <c r="N70" t="n">
+        <v>0.6366116568638961</v>
+      </c>
+      <c r="O70" t="n">
+        <v>0.7923998388587306</v>
+      </c>
+      <c r="P70" t="n">
+        <v>0.3564688723659779</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>0.680671052102248</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>val_snowy</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>0.47318</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.30775</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0.31006</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0.13296</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0.36479</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0.49007</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0.13762</v>
+      </c>
+      <c r="L71" t="n">
+        <v>0.41329</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0.30682</v>
+      </c>
+      <c r="N71" t="n">
+        <v>0.47523</v>
+      </c>
+      <c r="O71" t="n">
+        <v>0.79331</v>
+      </c>
+      <c r="P71" t="n">
+        <v>0.22772</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>0.56284</v>
+      </c>
+      <c r="R71" t="n">
+        <v>0.08423</v>
+      </c>
+      <c r="S71" t="n">
+        <v>0.39042</v>
+      </c>
+      <c r="T71" t="n">
+        <v>0.49414</v>
+      </c>
+      <c r="U71" t="n">
+        <v>0.11881</v>
+      </c>
+      <c r="V71" t="n">
+        <v>0.46269</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:22:31.350082+07:00</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>set1_night_aug</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>val_snowy</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>0.5173778856621206</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.3281296216521216</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0.1315626446900324</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0.4122131760561643</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0.4995188543685071</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0.1272340301974448</v>
+      </c>
+      <c r="L72" t="n">
+        <v>0.4701194029484593</v>
+      </c>
+      <c r="M72" t="n">
+        <v>0.3155134668037072</v>
+      </c>
+      <c r="N72" t="n">
+        <v>0.540885426911617</v>
+      </c>
+      <c r="O72" t="n">
+        <v>0.8004842235220488</v>
+      </c>
+      <c r="P72" t="n">
+        <v>0.2866114982578397</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>0.6433948128153902</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>val_clear</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>0.55393</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0.34428</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0.34691</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0.23029</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0.42098</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0.45888</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0.19472</v>
+      </c>
+      <c r="L73" t="n">
+        <v>0.41655</v>
+      </c>
+      <c r="M73" t="n">
+        <v>0.46726</v>
+      </c>
+      <c r="N73" t="n">
+        <v>0.54273</v>
+      </c>
+      <c r="O73" t="n">
+        <v>0.77882</v>
+      </c>
+      <c r="P73" t="n">
+        <v>0.41884</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>0.56203</v>
+      </c>
+      <c r="R73" t="n">
+        <v>0.19334</v>
+      </c>
+      <c r="S73" t="n">
+        <v>0.48169</v>
+      </c>
+      <c r="T73" t="n">
+        <v>0.44777</v>
+      </c>
+      <c r="U73" t="n">
+        <v>0.14403</v>
+      </c>
+      <c r="V73" t="n">
+        <v>0.46773</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>val_clear</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>0.5810641560126374</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0.3652510555971555</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0.2291323776458888</v>
+      </c>
+      <c r="I74" t="n">
+        <v>0.473811591848628</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0.4668978624282261</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0.2010019283054882</v>
+      </c>
+      <c r="L74" t="n">
+        <v>0.4554115177575464</v>
+      </c>
+      <c r="M74" t="n">
+        <v>0.4622974828721279</v>
+      </c>
+      <c r="N74" t="n">
+        <v>0.6173591720542971</v>
+      </c>
+      <c r="O74" t="n">
+        <v>0.782308814848631</v>
+      </c>
+      <c r="P74" t="n">
+        <v>0.426391668832411</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>0.6169636414557199</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>val_foggy</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>0.64608</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0.27821</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0.2242</v>
+      </c>
+      <c r="H75" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I75" t="n">
+        <v>-1</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0.44751</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L75" t="n">
+        <v>0.18713</v>
+      </c>
+      <c r="M75" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N75" t="n">
+        <v>-1</v>
+      </c>
+      <c r="O75" t="n">
+        <v>0.73032</v>
+      </c>
+      <c r="P75" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>0.20792</v>
+      </c>
+      <c r="R75" t="n">
+        <v>-1</v>
+      </c>
+      <c r="S75" t="n">
+        <v>-1</v>
+      </c>
+      <c r="T75" t="n">
+        <v>0.46469</v>
+      </c>
+      <c r="U75" t="n">
+        <v>0</v>
+      </c>
+      <c r="V75" t="n">
+        <v>0.20792</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>val_foggy</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>0.6621317587973919</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0.2582119023816812</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0.4549298247921024</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0.09950000000000001</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0.2202058823529412</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0.725807041098058</v>
+      </c>
+      <c r="P76" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>0.2655882352941177</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>val_overcast</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>0.56194</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.35073</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0.3463</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0.2473</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0.41185</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0.51197</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0.14407</v>
+      </c>
+      <c r="L77" t="n">
+        <v>0.43845</v>
+      </c>
+      <c r="M77" t="n">
+        <v>0.52685</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0.54155</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0.8138300000000001</v>
+      </c>
+      <c r="P77" t="n">
+        <v>0.31447</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>0.613</v>
+      </c>
+      <c r="R77" t="n">
+        <v>0.17903</v>
+      </c>
+      <c r="S77" t="n">
+        <v>0.44194</v>
+      </c>
+      <c r="T77" t="n">
+        <v>0.517</v>
+      </c>
+      <c r="U77" t="n">
+        <v>0.11095</v>
+      </c>
+      <c r="V77" t="n">
+        <v>0.48259</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>val_overcast</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>0.5973381607698339</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0.373132846175705</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.2489030086488966</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0.4588368745695126</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0.5212453641413004</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0.1652674277385882</v>
+      </c>
+      <c r="L78" t="n">
+        <v>0.4714115557802273</v>
+      </c>
+      <c r="M78" t="n">
+        <v>0.5194252400827171</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0.6113818296047231</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0.8197915946746285</v>
+      </c>
+      <c r="P78" t="n">
+        <v>0.3843594965261944</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>0.6517326429609063</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>val_partlycloudy</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>0.54793</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0.3597</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0.3678</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0.18765</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0.45287</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0.49404</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0.22009</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0.44385</v>
+      </c>
+      <c r="M79" t="n">
+        <v>0.37268</v>
+      </c>
+      <c r="N79" t="n">
+        <v>0.59398</v>
+      </c>
+      <c r="O79" t="n">
+        <v>0.79174</v>
+      </c>
+      <c r="P79" t="n">
+        <v>0.37757</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>0.6036899999999999</v>
+      </c>
+      <c r="R79" t="n">
+        <v>0.16555</v>
+      </c>
+      <c r="S79" t="n">
+        <v>0.47968</v>
+      </c>
+      <c r="T79" t="n">
+        <v>0.49791</v>
+      </c>
+      <c r="U79" t="n">
+        <v>0.22396</v>
+      </c>
+      <c r="V79" t="n">
+        <v>0.47192</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>val_partlycloudy</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>0.5779858331133153</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0.3778142410014214</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0.1859679829597952</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0.4857576306018299</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0.5022043166472543</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0.234200243124654</v>
+      </c>
+      <c r="L80" t="n">
+        <v>0.4809410316735738</v>
+      </c>
+      <c r="M80" t="n">
+        <v>0.4036690768893031</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0.6451513750485991</v>
+      </c>
+      <c r="O80" t="n">
+        <v>0.7963579782204812</v>
+      </c>
+      <c r="P80" t="n">
+        <v>0.3955516970961057</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>0.6491990383120874</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>val_rainy</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>0.5503400000000001</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0.36336</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0.38705</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0.25193</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0.41188</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0.48721</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0.21968</v>
+      </c>
+      <c r="L81" t="n">
+        <v>0.44611</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0.48904</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0.52862</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0.7938499999999999</v>
+      </c>
+      <c r="P81" t="n">
+        <v>0.31781</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>0.6224</v>
+      </c>
+      <c r="R81" t="n">
+        <v>0.24386</v>
+      </c>
+      <c r="S81" t="n">
+        <v>0.44665</v>
+      </c>
+      <c r="T81" t="n">
+        <v>0.48948</v>
+      </c>
+      <c r="U81" t="n">
+        <v>0.25472</v>
+      </c>
+      <c r="V81" t="n">
+        <v>0.50053</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>val_rainy</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>0.5850399335507009</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0.3849116834322024</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0.2499413104537883</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0.4683130330856607</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0.4961418435404604</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0.2167871763398219</v>
+      </c>
+      <c r="L82" t="n">
+        <v>0.4933750537412805</v>
+      </c>
+      <c r="M82" t="n">
+        <v>0.4809545303711791</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0.6105714067983378</v>
+      </c>
+      <c r="O82" t="n">
+        <v>0.7943336962253956</v>
+      </c>
+      <c r="P82" t="n">
+        <v>0.349239353803718</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>0.6901006805548742</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>val_snowy</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>pycocotools</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>0.48125</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0.31344</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0.32193</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0.13923</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0.36745</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0.48912</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0.1505</v>
+      </c>
+      <c r="L83" t="n">
+        <v>0.4209</v>
+      </c>
+      <c r="M83" t="n">
+        <v>0.33119</v>
+      </c>
+      <c r="N83" t="n">
+        <v>0.46862</v>
+      </c>
+      <c r="O83" t="n">
+        <v>0.79754</v>
+      </c>
+      <c r="P83" t="n">
+        <v>0.22772</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>0.58118</v>
+      </c>
+      <c r="R83" t="n">
+        <v>0.11343</v>
+      </c>
+      <c r="S83" t="n">
+        <v>0.41317</v>
+      </c>
+      <c r="T83" t="n">
+        <v>0.49212</v>
+      </c>
+      <c r="U83" t="n">
+        <v>0.11881</v>
+      </c>
+      <c r="V83" t="n">
+        <v>0.47214</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-10-09T21:28:00.329076+07:00</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>set3_combined</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>val_snowy</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ultralytics</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>0.5195750767434995</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0.3394036552800826</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0.1409800157431148</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0.4158481402870826</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0.4986010552997707</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0.1708746291468129</v>
+      </c>
+      <c r="L84" t="n">
+        <v>0.4707144359236317</v>
+      </c>
+      <c r="M84" t="n">
+        <v>0.3293884907898236</v>
+      </c>
+      <c r="N84" t="n">
+        <v>0.5476017921878117</v>
+      </c>
+      <c r="O84" t="n">
+        <v>0.8020982501037217</v>
+      </c>
+      <c r="P84" t="n">
+        <v>0.2778564685786209</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>0.6409303820575187</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>